<commit_message>
Refina layout e textos do diagnóstico guiado
</commit_message>
<xml_diff>
--- a/01 - DB/Base_Pai_Troubleshooting_Alertas_Falhas_MVP.xlsx
+++ b/01 - DB/Base_Pai_Troubleshooting_Alertas_Falhas_MVP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wesley\Documents\13 - TroubleShooting\01 - DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{143D9420-6E17-44BD-A271-3343C8CAA1B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDEA00C4-B30F-4749-8F31-3A21DEE0BD95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Instrucoes" sheetId="1" r:id="rId1"/>
@@ -473,9 +473,6 @@
     <t>Localização do sensor de pressão de Linha.</t>
   </si>
   <si>
-    <t>imagens/compressor/sensor_temp_compressor.jpg</t>
-  </si>
-  <si>
     <t>Documento de referência para inspeção do Sensor de temperatura do compressor.</t>
   </si>
   <si>
@@ -584,12 +581,6 @@
     <t>A falha FST003 está relacionada à temperatura do compressor acima de 115 °C?</t>
   </si>
   <si>
-    <t>Iniciar pelo PASSO 1.</t>
-  </si>
-  <si>
-    <t>Verificar se o código/variável selecionado está correto.</t>
-  </si>
-  <si>
     <t>FST003-P1</t>
   </si>
   <si>
@@ -623,12 +614,6 @@
     <t>A temperatura real do compressor está acima de 115 °C ou a tendência de temperatura confirma sobreaquecimento?</t>
   </si>
   <si>
-    <t>Prosseguir para inspeção do sistema de arrefecimento.</t>
-  </si>
-  <si>
-    <t>Investigar sensor, chicote, alimentação/sinal e leitura no PLC antes de atuar mecanicamente.</t>
-  </si>
-  <si>
     <t>FST003-P2</t>
   </si>
   <si>
@@ -662,12 +647,6 @@
     <t>Há conector solto, chicote danificado, mau contato, umidade, oxidação ou leitura elétrica incoerente?</t>
   </si>
   <si>
-    <t>Corrigir conexão/chicote/sensor e validar novamente.</t>
-  </si>
-  <si>
-    <t>Prosseguir para diagnóstico térmico/mecânico.</t>
-  </si>
-  <si>
     <t>FST003-P6</t>
   </si>
   <si>
@@ -698,12 +677,6 @@
     <t>A hélice está operando corretamente, sem danos/ruídos e com rotação adequada?</t>
   </si>
   <si>
-    <t>Prosseguir para inspeção do radiador/colmeia.</t>
-  </si>
-  <si>
-    <t>Corrigir sistema de acionamento da hélice.</t>
-  </si>
-  <si>
     <t>FST003-P3</t>
   </si>
   <si>
@@ -737,12 +710,6 @@
     <t>Há vazamento, pressão insuficiente ou falha no acionamento do motor da hélice?</t>
   </si>
   <si>
-    <t>Corrigir vazamento/pressão/acionamento e validar.</t>
-  </si>
-  <si>
-    <t>Prosseguir para limpeza e avaliação do radiador.</t>
-  </si>
-  <si>
     <t>Reparar vazamentos, mangueiras, conexões, motor hidráulico, bomba ou ajuste hidráulico conforme análise.</t>
   </si>
   <si>
@@ -770,12 +737,6 @@
     <t>O radiador/colmeia estava obstruído ou apresenta distribuição térmica anormal?</t>
   </si>
   <si>
-    <t>Realizar limpeza/correção da falha e validar temperatura.</t>
-  </si>
-  <si>
-    <t>Prosseguir para nível/condição do óleo do compressor.</t>
-  </si>
-  <si>
     <t>FST003-P4</t>
   </si>
   <si>
@@ -806,12 +767,6 @@
     <t>O nível/condição do óleo está fora do especificado ou há indício de contaminação/saturação?</t>
   </si>
   <si>
-    <t>Corrigir nível/óleo/filtros e validar.</t>
-  </si>
-  <si>
-    <t>Prosseguir para admissão de ar da unidade compressora.</t>
-  </si>
-  <si>
     <t>FST003-P5</t>
   </si>
   <si>
@@ -839,12 +794,6 @@
     <t>Inspecionar filtro de admissão de ar, tubulação de admissão, válvula gaveta com presença de pó e filtro separador no reservatório de ar.</t>
   </si>
   <si>
-    <t>Corrigir restrição e validar operação.</t>
-  </si>
-  <si>
-    <t>Prosseguir para inspeção interna/especializada da unidade compressora.</t>
-  </si>
-  <si>
     <t>FST003-P5A</t>
   </si>
   <si>
@@ -875,9 +824,6 @@
     <t>Há indício de dano interno na unidade compressora?</t>
   </si>
   <si>
-    <t>Executar validação final e monitoramento.</t>
-  </si>
-  <si>
     <t>Manutenção especializada</t>
   </si>
   <si>
@@ -908,9 +854,6 @@
     <t>A falha permanece inativa e a temperatura fica abaixo do limite durante o teste?</t>
   </si>
   <si>
-    <t>Reparo concluído. Registrar evidências e liberar máquina.</t>
-  </si>
-  <si>
     <t>Concluir</t>
   </si>
   <si>
@@ -971,12 +914,6 @@
     <t>Há filtro/tubulação/válvula obstruída ou filtro separador saturado?</t>
   </si>
   <si>
-    <t>Encaminhar para manutenção especializada/Departamento Técnico.</t>
-  </si>
-  <si>
-    <t>Retornar ao passo compatível com o sintoma observado ou escalar para Departamento Técnico.</t>
-  </si>
-  <si>
     <t>Localização do sensor de Temperatura do Óleo Hidráulico.</t>
   </si>
   <si>
@@ -993,6 +930,69 @@
   </si>
   <si>
     <t>imagens/percussão/sensor_pressao_percussao.jpg</t>
+  </si>
+  <si>
+    <t>Base confirmada. Iniciar o diagnóstico pelo Passo 1.</t>
+  </si>
+  <si>
+    <t>Código ou condição não compatível. Revisar o código da falha antes de usar este roteiro.</t>
+  </si>
+  <si>
+    <t>Falha real confirmada. Não substituir componentes ainda; prosseguir para inspeção do sistema de arrefecimento.</t>
+  </si>
+  <si>
+    <t>Falha real não confirmada ou leitura incoerente. Verificar sensor, chicote, alimentação/sinal e leitura no PLC antes de atuar mecanicamente.</t>
+  </si>
+  <si>
+    <t>Falha elétrica/instrumentação encontrada. Corrigir conexão, chicote ou sensor; validar a leitura e só então avançar para a validação final.</t>
+  </si>
+  <si>
+    <t>Nenhuma falha elétrica evidente. Não aplicar reparo neste ponto; prosseguir para diagnóstico térmico/mecânico.</t>
+  </si>
+  <si>
+    <t>Hélice operando corretamente. Não aplicar reparo neste ponto; prosseguir para inspeção do radiador/colmeia.</t>
+  </si>
+  <si>
+    <t>Condição reprovada. Corrigir danos mecânicos evidentes da hélice; se a suspeita for acionamento hidráulico, avançar para o subpasso P2A antes de concluir o reparo.</t>
+  </si>
+  <si>
+    <t>Falha hidráulica confirmada. Corrigir vazamento, pressão ou acionamento; validar o funcionamento da hélice e só então avançar para a validação final.</t>
+  </si>
+  <si>
+    <t>Sem falha hidráulica evidente. Não aplicar reparo neste ponto; prosseguir para limpeza e avaliação do radiador.</t>
+  </si>
+  <si>
+    <t>Obstrução ou troca térmica anormal encontrada. Limpar/corrigir o radiador/colmeia, validar a temperatura e só então avançar para a validação final.</t>
+  </si>
+  <si>
+    <t>Radiador/colmeia sem anomalia relevante. Não aplicar reparo neste ponto; prosseguir para verificação do nível e condição do óleo.</t>
+  </si>
+  <si>
+    <t>Óleo, nível ou filtros fora do especificado. Corrigir nível, óleo e filtros; validar a operação e só então avançar para a validação final.</t>
+  </si>
+  <si>
+    <t>Óleo e nível dentro do especificado. Não aplicar reparo neste ponto; prosseguir para verificação da admissão de ar da unidade compressora.</t>
+  </si>
+  <si>
+    <t>Restrição ou saturação encontrada. Corrigir admissão, tubulação, válvula ou filtro separador; validar a operação e só então avançar para a validação final.</t>
+  </si>
+  <si>
+    <t>Admissão e filtro separador sem anomalia evidente. Não aplicar reparo neste ponto; prosseguir para inspeção interna/especializada da unidade compressora.</t>
+  </si>
+  <si>
+    <t>Indício de dano interno encontrado. Não executar reparo em campo nem liberar a máquina; encaminhar para manutenção especializada/Departamento Técnico.</t>
+  </si>
+  <si>
+    <t>Sem indício de dano interno. Nenhum reparo interno necessário neste ponto; executar validação final e monitoramento.</t>
+  </si>
+  <si>
+    <t>Falha inativa e temperatura normalizada. Registrar evidências do teste e liberar a máquina.</t>
+  </si>
+  <si>
+    <t>Falha recorrente ou temperatura ainda elevada. Não liberar a máquina; retornar ao passo compatível com o sintoma observado ou escalar para o Departamento Técnico.</t>
+  </si>
+  <si>
+    <t>imagens\compressor\Sensor temperatura do compressor Ligação - 00.jpeg</t>
   </si>
 </sst>
 </file>
@@ -1286,16 +1286,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1307,196 +1310,38 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="88">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Carlito"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF666666"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF274E13"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9EAD3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF38761D"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF990000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF666666"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF274E13"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9EAD3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF38761D"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF990000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="76">
     <dxf>
       <font>
         <color rgb="FF666666"/>
@@ -1559,84 +1404,45 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor theme="1"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Carlito"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1773,6 +1579,78 @@
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1787,67 +1665,67 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TabelaTroubleshooting" displayName="TabelaTroubleshooting" ref="A1:T194" headerRowDxfId="87" dataDxfId="86" totalsRowDxfId="85">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TabelaTroubleshooting" displayName="TabelaTroubleshooting" ref="A1:T194" headerRowDxfId="51" dataDxfId="50" totalsRowDxfId="49">
   <tableColumns count="20">
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Código" dataDxfId="84"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Tipo" dataDxfId="83"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Sistema" dataDxfId="82"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Subsistema" dataDxfId="81"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Severidade" dataDxfId="80"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Prioridade" dataDxfId="79"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Status" dataDxfId="78"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Mensagem na IHM / Alerta" dataDxfId="77"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Descrição resumida" dataDxfId="76"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Causa" dataDxfId="75"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Efeito na máquina/operação" dataDxfId="74"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Solução" dataDxfId="73"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Validação após solução" dataDxfId="72"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Origem" dataDxfId="71"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Variável / Código relacionado" dataDxfId="70"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Ferramentas necessárias" dataDxfId="69"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Observações" dataDxfId="68"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Responsável" dataDxfId="67"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Data revisão" dataDxfId="66"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Versão" dataDxfId="65"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Código" dataDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Tipo" dataDxfId="47"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Sistema" dataDxfId="46"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Subsistema" dataDxfId="45"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Severidade" dataDxfId="44"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Prioridade" dataDxfId="43"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Status" dataDxfId="42"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Mensagem na IHM / Alerta" dataDxfId="41"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Descrição resumida" dataDxfId="40"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Causa" dataDxfId="39"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Efeito na máquina/operação" dataDxfId="38"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Solução" dataDxfId="37"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Validação após solução" dataDxfId="36"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Origem" dataDxfId="35"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Variável / Código relacionado" dataDxfId="34"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Ferramentas necessárias" dataDxfId="33"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Observações" dataDxfId="32"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Responsável" dataDxfId="31"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Data revisão" dataDxfId="30"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Versão" dataDxfId="29"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{20343510-14AE-4192-A250-078DD82C5713}" name="TabelaDiagnosticoGuiado7" displayName="TabelaDiagnosticoGuiado7" ref="A1:O149" headerRowDxfId="45" dataDxfId="44" totalsRowDxfId="43">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{20343510-14AE-4192-A250-078DD82C5713}" name="TabelaDiagnosticoGuiado7" displayName="TabelaDiagnosticoGuiado7" ref="A1:O149" headerRowDxfId="75" dataDxfId="74" totalsRowDxfId="73">
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{63450B7D-49ED-41CF-B7D9-D287ED2CF298}" name="Código Item" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{46817399-D7BC-4925-942C-4CBCE861CEFB}" name="ID Passo" dataDxfId="41"/>
-    <tableColumn id="6" xr3:uid="{928114F4-FCAD-4C37-A4EF-819E9DF70EE8}" name="Nível" dataDxfId="40"/>
-    <tableColumn id="10" xr3:uid="{0D5C296C-DF81-40F3-8730-12258FC5A1C2}" name="Título do passo" dataDxfId="39"/>
-    <tableColumn id="13" xr3:uid="{C4B409B0-4E84-4D56-99DA-C47BE047C82F}" name="Condições" dataDxfId="38"/>
-    <tableColumn id="7" xr3:uid="{47B506C2-F1DC-4C47-B635-B1053D535C32}" name="Ação" dataDxfId="37"/>
-    <tableColumn id="8" xr3:uid="{9A1FD092-B7F8-4418-972E-572CF38F7734}" name="Especificação / Pergunta" dataDxfId="36"/>
-    <tableColumn id="12" xr3:uid="{79AF0F65-1615-411F-8D61-AF8DFB68EDBF}" name="Se SIM / OK" dataDxfId="35"/>
-    <tableColumn id="9" xr3:uid="{CE6BA67B-F888-46B1-8996-7107D16FBC60}" name="Se NÃO / NOK" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{22956E1A-E929-4E4C-96B4-A516DE98DA89}" name="Próximo passo SIM" dataDxfId="32" totalsRowDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{D666DC4B-08B4-4658-ADE8-914DB4BD8A6F}" name="Próximo passo NÃO" dataDxfId="30" totalsRowDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{6B4D0F42-A199-4F72-BCF8-87057820DA0B}" name="Reparo / Correção" dataDxfId="28" totalsRowDxfId="29"/>
-    <tableColumn id="11" xr3:uid="{B3E9C756-122E-4985-8678-E9E7E5C73523}" name="Ferramentas" dataDxfId="26" totalsRowDxfId="27"/>
-    <tableColumn id="14" xr3:uid="{98C258F9-4844-4EE4-A584-C7C40BA218E3}" name="Segurança" dataDxfId="24" totalsRowDxfId="25"/>
-    <tableColumn id="15" xr3:uid="{9450BD72-74B1-4478-982C-C7612EE8B7EC}" name="Observações" dataDxfId="22" totalsRowDxfId="23"/>
+    <tableColumn id="1" xr3:uid="{63450B7D-49ED-41CF-B7D9-D287ED2CF298}" name="Código Item" dataDxfId="72"/>
+    <tableColumn id="4" xr3:uid="{46817399-D7BC-4925-942C-4CBCE861CEFB}" name="ID Passo" dataDxfId="71"/>
+    <tableColumn id="6" xr3:uid="{928114F4-FCAD-4C37-A4EF-819E9DF70EE8}" name="Nível" dataDxfId="70"/>
+    <tableColumn id="10" xr3:uid="{0D5C296C-DF81-40F3-8730-12258FC5A1C2}" name="Título do passo" dataDxfId="69"/>
+    <tableColumn id="13" xr3:uid="{C4B409B0-4E84-4D56-99DA-C47BE047C82F}" name="Condições" dataDxfId="68"/>
+    <tableColumn id="7" xr3:uid="{47B506C2-F1DC-4C47-B635-B1053D535C32}" name="Ação" dataDxfId="67"/>
+    <tableColumn id="8" xr3:uid="{9A1FD092-B7F8-4418-972E-572CF38F7734}" name="Especificação / Pergunta" dataDxfId="66"/>
+    <tableColumn id="12" xr3:uid="{79AF0F65-1615-411F-8D61-AF8DFB68EDBF}" name="Se SIM / OK" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{CE6BA67B-F888-46B1-8996-7107D16FBC60}" name="Se NÃO / NOK" dataDxfId="64"/>
+    <tableColumn id="2" xr3:uid="{22956E1A-E929-4E4C-96B4-A516DE98DA89}" name="Próximo passo SIM" dataDxfId="63" totalsRowDxfId="62"/>
+    <tableColumn id="3" xr3:uid="{D666DC4B-08B4-4658-ADE8-914DB4BD8A6F}" name="Próximo passo NÃO" dataDxfId="61" totalsRowDxfId="60"/>
+    <tableColumn id="5" xr3:uid="{6B4D0F42-A199-4F72-BCF8-87057820DA0B}" name="Reparo / Correção" dataDxfId="59" totalsRowDxfId="58"/>
+    <tableColumn id="11" xr3:uid="{B3E9C756-122E-4985-8678-E9E7E5C73523}" name="Ferramentas" dataDxfId="57" totalsRowDxfId="56"/>
+    <tableColumn id="14" xr3:uid="{98C258F9-4844-4EE4-A584-C7C40BA218E3}" name="Segurança" dataDxfId="55" totalsRowDxfId="54"/>
+    <tableColumn id="15" xr3:uid="{9450BD72-74B1-4478-982C-C7612EE8B7EC}" name="Observações" dataDxfId="53" totalsRowDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="TabelaAnexos" displayName="TabelaAnexos" ref="A1:H150" headerRowDxfId="64" dataDxfId="63" totalsRowDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="TabelaAnexos" displayName="TabelaAnexos" ref="A1:H150" headerRowDxfId="28" dataDxfId="27" totalsRowDxfId="26">
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="ID Anexo" dataDxfId="61"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="ID Falha/Alerta" dataDxfId="60"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Tipo" dataDxfId="59"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Título" dataDxfId="58"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Arquivo/Caminho relativo" dataDxfId="57"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Descrição" dataDxfId="56"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="Ordem" dataDxfId="55"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="Observações" dataDxfId="54"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="ID Anexo" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="ID Falha/Alerta" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Tipo" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Título" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Arquivo/Caminho relativo" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Descrição" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="Ordem" dataDxfId="19"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="Observações" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1856,31 +1734,31 @@
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E7FB7C67-C65F-4505-9C4D-61650793003B}" name="TabelaRevisoes8" displayName="TabelaRevisoes8" ref="A1:G100">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{887893B9-5C05-462C-B28A-8A617572CDF7}" name="Versão" dataDxfId="53"/>
-    <tableColumn id="2" xr3:uid="{2C793684-7A8D-471D-8CBE-D9532CB77901}" name="Data" dataDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{000059D5-04B3-4C9E-B6AF-D65E3727CCF2}" name="Responsável" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{12B4137F-2367-4A0F-842C-C89186E2354B}" name="Tipo alteração" dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{A13506EB-4C05-4057-8105-5C301E7D91EA}" name="Descrição" dataDxfId="49"/>
-    <tableColumn id="6" xr3:uid="{2AADEF3D-2C85-4C01-AC94-A8E880A6DE51}" name="Itens alterados" dataDxfId="48"/>
-    <tableColumn id="7" xr3:uid="{4993FF7B-FBFE-4ECE-B9DA-5E29E3DC50CC}" name="Status publicação" dataDxfId="47"/>
+    <tableColumn id="1" xr3:uid="{887893B9-5C05-462C-B28A-8A617572CDF7}" name="Versão" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{2C793684-7A8D-471D-8CBE-D9532CB77901}" name="Data" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{000059D5-04B3-4C9E-B6AF-D65E3727CCF2}" name="Responsável" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{12B4137F-2367-4A0F-842C-C89186E2354B}" name="Tipo alteração" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{A13506EB-4C05-4057-8105-5C301E7D91EA}" name="Descrição" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{2AADEF3D-2C85-4C01-AC94-A8E880A6DE51}" name="Itens alterados" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{4993FF7B-FBFE-4ECE-B9DA-5E29E3DC50CC}" name="Status publicação" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{3DB27BD3-6A2F-4D61-AC70-8EE0764C8E29}" name="Tabela6" displayName="Tabela6" ref="A1:B9" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{3DB27BD3-6A2F-4D61-AC70-8EE0764C8E29}" name="Tabela6" displayName="Tabela6" ref="A1:B9" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="A1:B9" xr:uid="{3DB27BD3-6A2F-4D61-AC70-8EE0764C8E29}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{3E53F907-59F0-473F-9398-6A2A04970646}" name="Campo / Seção" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{AAF21FA1-7E9C-44E5-BD1B-108C6C417EE8}" name="Definição aplicada no documento" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{3E53F907-59F0-473F-9398-6A2A04970646}" name="Campo / Seção" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{AAF21FA1-7E9C-44E5-BD1B-108C6C417EE8}" name="Definição aplicada no documento" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="TabelaListas" displayName="TabelaListas" ref="A1:H17" headerRowDxfId="46">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="TabelaListas" displayName="TabelaListas" ref="A1:H17" headerRowDxfId="6">
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Tipo"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Sistema"/>
@@ -2053,270 +1931,270 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21.6" thickBot="1">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="23"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="16"/>
     </row>
     <row r="2" spans="1:8" ht="14.4" thickBot="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="19"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="20"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="22"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="13"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="25"/>
     </row>
     <row r="5" spans="1:8" ht="14.4" thickBot="1">
       <c r="A5" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="15"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="28"/>
     </row>
     <row r="6" spans="1:8" ht="14.4" thickBot="1">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="18"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="19"/>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="20"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="22"/>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="13"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="25"/>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="13"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="25"/>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="13"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="25"/>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="13"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="25"/>
     </row>
     <row r="12" spans="1:8" ht="14.4" thickBot="1">
       <c r="A12" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="15"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="28"/>
     </row>
     <row r="13" spans="1:8" ht="14.4" thickBot="1">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="18"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="19"/>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="20"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="22"/>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="13"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="25"/>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="13"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="25"/>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="13"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="25"/>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="13"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="25"/>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="13"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="24"/>
+      <c r="H19" s="25"/>
     </row>
     <row r="20" spans="1:8" ht="14.4" thickBot="1">
       <c r="A20" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="15"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="28"/>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="3"/>
@@ -2340,26 +2218,26 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B19:H19"/>
+    <mergeCell ref="B20:H20"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="B8:H8"/>
+    <mergeCell ref="B9:H9"/>
+    <mergeCell ref="B10:H10"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="B7:H7"/>
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="B9:H9"/>
-    <mergeCell ref="B10:H10"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B15:H15"/>
-    <mergeCell ref="B16:H16"/>
-    <mergeCell ref="B17:H17"/>
-    <mergeCell ref="B18:H18"/>
-    <mergeCell ref="B19:H19"/>
-    <mergeCell ref="B20:H20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2451,7 +2329,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="124.2">
+    <row r="2" spans="1:20" ht="110.4">
       <c r="A2" s="3" t="s">
         <v>114</v>
       </c>
@@ -2462,7 +2340,7 @@
         <v>94</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>55</v>
@@ -2477,40 +2355,40 @@
         <v>123</v>
       </c>
       <c r="I2" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="J2" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>159</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>160</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>117</v>
       </c>
       <c r="P2" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="Q2" s="3" t="s">
         <v>161</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>162</v>
       </c>
       <c r="R2" s="3" t="s">
         <v>52</v>
       </c>
       <c r="S2" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="T2" s="3" t="s">
         <v>163</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:20" ht="12" customHeight="1">
@@ -6739,24 +6617,24 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E194">
-    <cfRule type="expression" dxfId="21" priority="1">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>E2="Crítica"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>E2="Alta"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="3">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>E2="Média"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="4">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>E2="Baixa"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G194">
-    <cfRule type="expression" dxfId="17" priority="5">
+    <cfRule type="expression" dxfId="1" priority="5">
       <formula>G2="Publicado"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="6">
+    <cfRule type="expression" dxfId="0" priority="6">
       <formula>G2="Rascunho"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6831,42 +6709,42 @@
     <col min="15" max="16384" width="47.5" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:15" ht="27.6">
       <c r="A1" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>60</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>173</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>174</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>63</v>
@@ -6883,46 +6761,46 @@
         <v>114</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="J2" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="O2" s="3" t="s">
         <v>185</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="41.4">
@@ -6930,46 +6808,46 @@
         <v>114</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="H3" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="J3" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="M3" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="N3" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="O3" s="3" t="s">
         <v>196</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="41.4">
@@ -6977,93 +6855,93 @@
         <v>114</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="K4" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="L4" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="M4" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="N4" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="O4" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="H4" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="N4" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" ht="41.4">
+    </row>
+    <row r="5" spans="1:15" ht="55.2">
       <c r="A5" s="3" t="s">
         <v>114</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="L5" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="M5" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="N5" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="O5" s="3" t="s">
         <v>217</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="N5" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="6" spans="1:15" ht="41.4">
@@ -7071,46 +6949,46 @@
         <v>114</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="G6" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>231</v>
-      </c>
       <c r="H6" s="3" t="s">
-        <v>232</v>
+        <v>305</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>233</v>
+        <v>306</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="55.2">
@@ -7118,46 +6996,46 @@
         <v>114</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>240</v>
+        <v>229</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>241</v>
+        <v>230</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>243</v>
+        <v>307</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>244</v>
+        <v>308</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>245</v>
+        <v>232</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>246</v>
+        <v>233</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>248</v>
+        <v>235</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>249</v>
+        <v>236</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="41.4">
@@ -7165,46 +7043,46 @@
         <v>114</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="N8" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>253</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>256</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>258</v>
-      </c>
-      <c r="M8" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="N8" s="3" t="s">
-        <v>260</v>
-      </c>
       <c r="O8" s="3" t="s">
-        <v>261</v>
+        <v>246</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="41.4">
@@ -7212,46 +7090,46 @@
         <v>114</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>257</v>
+        <v>242</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>262</v>
+        <v>247</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>263</v>
+        <v>248</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>264</v>
+        <v>249</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>265</v>
+        <v>250</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>309</v>
+        <v>290</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>266</v>
+        <v>311</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>267</v>
+        <v>312</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>268</v>
+        <v>251</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>269</v>
+        <v>252</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>270</v>
+        <v>253</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>271</v>
+        <v>254</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>272</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="41.4">
@@ -7259,93 +7137,93 @@
         <v>114</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>268</v>
+        <v>251</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>273</v>
+        <v>256</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>274</v>
+        <v>257</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>275</v>
+        <v>258</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>276</v>
+        <v>259</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>277</v>
+        <v>260</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>278</v>
+        <v>314</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>279</v>
+        <v>261</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>280</v>
+        <v>262</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>281</v>
+        <v>263</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>282</v>
+        <v>264</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" ht="41.4">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="55.2">
       <c r="A11" s="3" t="s">
         <v>114</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>284</v>
+        <v>266</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>285</v>
+        <v>267</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>286</v>
+        <v>268</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>287</v>
+        <v>269</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>288</v>
+        <v>270</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>289</v>
+        <v>315</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>290</v>
+        <v>271</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>291</v>
+        <v>272</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>292</v>
+        <v>273</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>293</v>
+        <v>274</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>294</v>
+        <v>275</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>295</v>
+        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -7412,10 +7290,10 @@
         <v>138</v>
       </c>
       <c r="E2" s="11" t="s">
+        <v>317</v>
+      </c>
+      <c r="F2" s="11" t="s">
         <v>144</v>
-      </c>
-      <c r="F2" s="11" t="s">
-        <v>145</v>
       </c>
       <c r="G2" s="3">
         <v>1</v>
@@ -7435,13 +7313,13 @@
         <v>73</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>312</v>
+        <v>291</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>313</v>
+        <v>292</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>314</v>
+        <v>293</v>
       </c>
       <c r="G3" s="3">
         <v>1</v>
@@ -7464,10 +7342,10 @@
         <v>139</v>
       </c>
       <c r="E4" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="F4" s="11" t="s">
         <v>146</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>147</v>
       </c>
       <c r="G4" s="3">
         <v>1</v>
@@ -7490,10 +7368,10 @@
         <v>140</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>315</v>
+        <v>294</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G5" s="3">
         <v>1</v>
@@ -7516,10 +7394,10 @@
         <v>141</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>316</v>
+        <v>295</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G6" s="3">
         <v>1</v>
@@ -7542,10 +7420,10 @@
         <v>142</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>317</v>
+        <v>296</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G7" s="3">
         <v>1</v>
@@ -7568,10 +7446,10 @@
         <v>143</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G8" s="3">
         <v>1</v>
@@ -10077,75 +9955,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="28" t="s">
-        <v>296</v>
-      </c>
-      <c r="B1" s="28" t="s">
-        <v>297</v>
+      <c r="A1" s="13" t="s">
+        <v>277</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="27.6">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="27" t="s">
-        <v>298</v>
+      <c r="B2" s="12" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="27.6">
-      <c r="A3" s="27" t="s">
-        <v>299</v>
-      </c>
-      <c r="B3" s="27" t="s">
-        <v>300</v>
+      <c r="A3" s="12" t="s">
+        <v>280</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="27.6">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="27" t="s">
-        <v>301</v>
+      <c r="B4" s="12" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="27.6">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="B5" s="27" t="s">
-        <v>302</v>
+      <c r="B5" s="12" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="27" t="s">
-        <v>174</v>
-      </c>
-      <c r="B6" s="27" t="s">
-        <v>303</v>
+      <c r="A6" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="27" t="s">
-        <v>304</v>
-      </c>
-      <c r="B7" s="27" t="s">
-        <v>305</v>
+      <c r="A7" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="27.6">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="27" t="s">
-        <v>306</v>
+      <c r="B8" s="12" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="27.6">
-      <c r="A9" s="27" t="s">
-        <v>307</v>
-      </c>
-      <c r="B9" s="27" t="s">
-        <v>308</v>
+      <c r="A9" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>289</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza tabela de anexos do troubleshooting
</commit_message>
<xml_diff>
--- a/01 - DB/Base_Pai_Troubleshooting_Alertas_Falhas_MVP.xlsx
+++ b/01 - DB/Base_Pai_Troubleshooting_Alertas_Falhas_MVP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wesley\Documents\13 - TroubleShooting\01 - DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDEA00C4-B30F-4749-8F31-3A21DEE0BD95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D3780D3-32BE-42CF-A04B-7F9D4907EACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Instrucoes" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="327">
   <si>
     <t>Base Pai - Troubleshooting de Alertas e Falhas</t>
   </si>
@@ -203,9 +203,6 @@
     <t>Alerta</t>
   </si>
   <si>
-    <t>Motor</t>
-  </si>
-  <si>
     <t>Crítica</t>
   </si>
   <si>
@@ -410,9 +407,6 @@
     <t>Linha</t>
   </si>
   <si>
-    <t>Alta temperatura compressor</t>
-  </si>
-  <si>
     <t>0.1.1</t>
   </si>
   <si>
@@ -458,9 +452,6 @@
     <t>Localização do sensor de Temperatura do compressor.</t>
   </si>
   <si>
-    <t>Localização do sensor de Temperatura do Motor.</t>
-  </si>
-  <si>
     <t>Localização do sensor de pressão do Avanço.</t>
   </si>
   <si>
@@ -476,9 +467,6 @@
     <t>Documento de referência para inspeção do Sensor de temperatura do compressor.</t>
   </si>
   <si>
-    <t>imagens/motor/sensor_temp_motor.jpg</t>
-  </si>
-  <si>
     <t>Documento de referência para inspeção do Sensor de temperatura do motor.</t>
   </si>
   <si>
@@ -503,24 +491,12 @@
     <t>Temperatura / Sistema de arrefecimento e lubrificação</t>
   </si>
   <si>
-    <t>Falha gerada quando a temperatura do compressor ultrapassa o limite permitido de operação.</t>
-  </si>
-  <si>
-    <t>Temperatura do compressor acima de 115 °C. A causa raiz deve ser confirmada no diagnóstico guiado: falha de arrefecimento, restrição no radiador/colmeia, ventilador/hélice sem desempenho, nível/condição de óleo inadequado, admissão restringida, filtro separador saturado, sensor/chicote com falha ou condição severa de operação.</t>
-  </si>
-  <si>
-    <t>Proteção da máquina por alta temperatura. Desligamento automático para evitar dano ao compressor.</t>
-  </si>
-  <si>
     <t>Executar o diagnóstico guiado FST003 e corrigir a causa raiz encontrada. Não tratar esta falha como uma única ação de troca. As ações possíveis incluem limpar o radiador/colmeia, corrigir hélice/acionamento hidráulico, normalizar nível e condição do óleo, corrigir sensor/chicote, remover restrições de admissão, substituir filtro separador/filtro de retorno/óleo quando aplicável e validar a temperatura em operação.</t>
   </si>
   <si>
     <t>Após o reparo, limpar/resetar a falha, operar a máquina em condição controlada, monitorar a temperatura do compressor na IHM/PLC/telemetria e confirmar que a temperatura permanece abaixo do limite de disparo e que a falha não retorna.</t>
   </si>
   <si>
-    <t>Sensor físico/Compressor</t>
-  </si>
-  <si>
     <t>IHM, PLC/CODESYS, telemetria, termômetro infravermelho, tacômetro, multímetro, kit de ferramentas, ferramentas de limpeza e EPI.</t>
   </si>
   <si>
@@ -914,12 +890,6 @@
     <t>Há filtro/tubulação/válvula obstruída ou filtro separador saturado?</t>
   </si>
   <si>
-    <t>Localização do sensor de Temperatura do Óleo Hidráulico.</t>
-  </si>
-  <si>
-    <t>imagens/hidráulico/sensor_temp_hidraulico.jpg</t>
-  </si>
-  <si>
     <t>Documento de referência para inspeção do Sensor de temperatura do óleo hidráulico.</t>
   </si>
   <si>
@@ -992,7 +962,64 @@
     <t>Falha recorrente ou temperatura ainda elevada. Não liberar a máquina; retornar ao passo compatível com o sintoma observado ou escalar para o Departamento Técnico.</t>
   </si>
   <si>
-    <t>imagens\compressor\Sensor temperatura do compressor Ligação - 00.jpeg</t>
+    <t>imagens\compressor\FOX 8-20 Sensor temperatura do compressor.jpeg</t>
+  </si>
+  <si>
+    <t>imagens\compressor\FOX 8-30 Sensor temperatura do compressor.jpeg</t>
+  </si>
+  <si>
+    <t>imagens\compressor\FOX 12-30C Sensor temperatura do compressor.jpeg</t>
+  </si>
+  <si>
+    <t>GVL_TX.FALHA_TEMP_HIDRAULICO</t>
+  </si>
+  <si>
+    <t>Temperatura / Sistema Hidráulico</t>
+  </si>
+  <si>
+    <t>Alta temperatura do Óleo Hidráulico</t>
+  </si>
+  <si>
+    <t>Falha gerada quando a temperatura do Óleo Hidráulico ultrapassa o limite permitido de operação.</t>
+  </si>
+  <si>
+    <t>Temperatura do Óleo Hidráulico acima de 100 °C.</t>
+  </si>
+  <si>
+    <t>Motor Diesel</t>
+  </si>
+  <si>
+    <t>Temperatura / Motor Diesel</t>
+  </si>
+  <si>
+    <t>Alta temperatura do Motor Diesel</t>
+  </si>
+  <si>
+    <t>Falha gerada quando a temperatura do Motor Diesel ultrapassa o limite permitido de operação.</t>
+  </si>
+  <si>
+    <t>Temperatura do Motor Diesel acima de 100 °C.</t>
+  </si>
+  <si>
+    <t>GVL_TX.FALHA_TEMP_MOTOR</t>
+  </si>
+  <si>
+    <t>Alta temperatura Compressor</t>
+  </si>
+  <si>
+    <t>Falha gerada quando a temperatura do Compressor ultrapassa o limite permitido de operação.</t>
+  </si>
+  <si>
+    <t>Temperatura do Compressor acima de 115 °C. A causa raiz deve ser confirmada no diagnóstico guiado: falha de arrefecimento, restrição no radiador/colmeia, ventilador/hélice sem desempenho, nível/condição de óleo inadequado, admissão restringida, filtro separador saturado, sensor/chicote com falha ou condição severa de operação.</t>
+  </si>
+  <si>
+    <t>Proteção da máquina por alta temperatura. Desligamento automático para evitar dano aos componentes Hidraulicos.</t>
+  </si>
+  <si>
+    <t>Proteção da máquina por alta temperatura. Desligamento automático para evitar dano ao Motor Diesel.</t>
+  </si>
+  <si>
+    <t>Proteção da máquina por alta temperatura. Desligamento automático para evitar dano ao Compressor.</t>
   </si>
 </sst>
 </file>
@@ -2331,109 +2358,173 @@
     </row>
     <row r="2" spans="1:20" ht="110.4">
       <c r="A2" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>47</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="H2" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="Q2" s="3" t="s">
         <v>153</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>161</v>
       </c>
       <c r="R2" s="3" t="s">
         <v>52</v>
       </c>
       <c r="S2" s="8" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" ht="12" customHeight="1">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" ht="49.2" customHeight="1">
+      <c r="A3" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>324</v>
+      </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-      <c r="O3" s="3"/>
+      <c r="N3" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>310</v>
+      </c>
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
-      <c r="S3" s="8"/>
-      <c r="T3" s="3"/>
-    </row>
-    <row r="4" spans="1:20" ht="12" customHeight="1">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
+      <c r="R3" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="S3" s="8">
+        <v>46149</v>
+      </c>
+      <c r="T3" s="3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" ht="41.4">
+      <c r="A4" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>325</v>
+      </c>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
+      <c r="N4" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>320</v>
+      </c>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="8"/>
-      <c r="T4" s="3"/>
+      <c r="R4" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="S4" s="8">
+        <v>46149</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="5" spans="1:20" ht="12" customHeight="1">
       <c r="A5" s="3"/>
@@ -6711,46 +6802,46 @@
   <sheetData>
     <row r="1" spans="1:15" ht="27.6">
       <c r="A1" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>173</v>
-      </c>
       <c r="M1" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="O1" s="3" t="s">
         <v>43</v>
@@ -6758,472 +6849,472 @@
     </row>
     <row r="2" spans="1:15" ht="27.6">
       <c r="A2" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="L2" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="O2" s="3" t="s">
         <v>177</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="41.4">
       <c r="A3" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="F3" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="M3" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="N3" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="O3" s="3" t="s">
         <v>188</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>300</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="41.4">
       <c r="A4" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="G4" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="N4" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="O4" s="3" t="s">
         <v>198</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>302</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="N4" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="55.2">
       <c r="A5" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="M5" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="N5" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="O5" s="3" t="s">
         <v>209</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>303</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>304</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="N5" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="6" spans="1:15" ht="41.4">
       <c r="A6" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="G6" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="O6" s="3" t="s">
         <v>218</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>305</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="L6" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="M6" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="N6" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="O6" s="3" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="55.2">
       <c r="A7" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="N7" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="O7" s="3" t="s">
         <v>228</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>231</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>307</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>308</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="M7" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="N7" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="O7" s="3" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="41.4">
       <c r="A8" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="G8" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="N8" s="3" t="s">
         <v>237</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="O8" s="3" t="s">
         <v>238</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>309</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>310</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="M8" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="N8" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="O8" s="3" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="41.4">
       <c r="A9" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="G9" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="M9" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="N9" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="O9" s="3" t="s">
         <v>247</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>290</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>311</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>312</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="M9" s="3" t="s">
-        <v>253</v>
-      </c>
-      <c r="N9" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="O9" s="3" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="41.4">
       <c r="A10" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="G10" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="N10" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="O10" s="3" t="s">
         <v>257</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>258</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>313</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="M10" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="N10" s="3" t="s">
-        <v>264</v>
-      </c>
-      <c r="O10" s="3" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="55.2">
       <c r="A11" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="M11" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="N11" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="O11" s="3" t="s">
         <v>268</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>270</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>315</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>272</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="M11" s="3" t="s">
-        <v>274</v>
-      </c>
-      <c r="N11" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="O11" s="3" t="s">
-        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -7252,25 +7343,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D1" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="F1" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F1" s="7" t="s">
-        <v>68</v>
-      </c>
       <c r="G1" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H1" s="7" t="s">
         <v>43</v>
@@ -7278,184 +7369,184 @@
     </row>
     <row r="2" spans="1:8" ht="27.6">
       <c r="A2" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="G2" s="3">
         <v>1</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="27.6">
       <c r="A3" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>73</v>
-      </c>
       <c r="D3" s="11" t="s">
-        <v>291</v>
+        <v>136</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>292</v>
+        <v>308</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>293</v>
+        <v>283</v>
       </c>
       <c r="G3" s="3">
         <v>1</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="27.6">
       <c r="A4" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>145</v>
+        <v>309</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="G4" s="3">
         <v>1</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="27.6">
       <c r="A5" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G5" s="3">
         <v>1</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="27.6">
       <c r="A6" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="G6" s="3">
         <v>1</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="27.6">
       <c r="A7" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G7" s="3">
         <v>1</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="27.6">
       <c r="A8" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="G8" s="3">
         <v>1</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -8886,7 +8977,7 @@
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0300-000000000000}">
           <x14:formula1>
             <xm:f>Listas!$H$2:$H$7</xm:f>
@@ -8918,27 +9009,27 @@
         <v>46</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>44</v>
       </c>
       <c r="D1" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="E1" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>76</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="27.6">
       <c r="A2" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B2" s="8">
         <v>46146</v>
@@ -8947,21 +9038,21 @@
         <v>52</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="27.6">
       <c r="A3" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B3" s="8">
         <v>46146</v>
@@ -8970,21 +9061,21 @@
         <v>52</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="E3" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="E3" s="11" t="s">
-        <v>127</v>
-      </c>
       <c r="F3" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="27.6">
       <c r="A4" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B4" s="8">
         <v>46146</v>
@@ -8993,21 +9084,21 @@
         <v>52</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="27.6">
       <c r="A5" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B5" s="8">
         <v>46146</v>
@@ -9016,21 +9107,21 @@
         <v>52</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="27.6">
       <c r="A6" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B6" s="8">
         <v>46146</v>
@@ -9039,21 +9130,21 @@
         <v>52</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="27.6">
       <c r="A7" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B7" s="8">
         <v>46146</v>
@@ -9062,21 +9153,21 @@
         <v>52</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="27.6">
       <c r="A8" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B8" s="8">
         <v>46146</v>
@@ -9085,16 +9176,16 @@
         <v>52</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -9956,10 +10047,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="13" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="27.6">
@@ -9967,15 +10058,15 @@
         <v>36</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="27.6">
       <c r="A3" s="12" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="27.6">
@@ -9983,31 +10074,31 @@
         <v>38</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="27.6">
       <c r="A5" s="12" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="12" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="12" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="27.6">
@@ -10015,15 +10106,15 @@
         <v>39</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="27.6">
       <c r="A9" s="12" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>
@@ -10062,10 +10153,10 @@
         <v>32</v>
       </c>
       <c r="G1" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="H1" s="7" t="s">
         <v>78</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="12" customHeight="1">
@@ -10073,25 +10164,25 @@
         <v>53</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>54</v>
+        <v>315</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>82</v>
-      </c>
       <c r="H2" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="12" customHeight="1">
@@ -10099,174 +10190,174 @@
         <v>47</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>50</v>
       </c>
       <c r="G3" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="12" customHeight="1">
       <c r="A4" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="E4" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="E4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="12" customHeight="1">
       <c r="A5" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>94</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>49</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>48</v>
       </c>
       <c r="F5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="H5" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="12" customHeight="1">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>100</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="12" customHeight="1">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H7" s="1" t="s">
         <v>105</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="12" customHeight="1">
       <c r="A8" s="1"/>
       <c r="B8" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H8" s="1"/>
     </row>
     <row r="9" spans="1:8" ht="12" customHeight="1">
       <c r="A9" s="1"/>
       <c r="B9" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H9" s="1"/>
     </row>
     <row r="10" spans="1:8" ht="12" customHeight="1">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H10" s="1"/>
     </row>
     <row r="11" spans="1:8" ht="12" customHeight="1">
       <c r="A11" s="1"/>
       <c r="B11" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
       <c r="G11" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H11" s="1"/>
     </row>
@@ -10280,14 +10371,14 @@
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H12" s="1"/>
     </row>
     <row r="13" spans="1:8" ht="12" customHeight="1">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -10299,7 +10390,7 @@
     <row r="14" spans="1:8" ht="12" customHeight="1">
       <c r="A14" s="1"/>
       <c r="B14" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -10311,7 +10402,7 @@
     <row r="15" spans="1:8" ht="12" customHeight="1">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -10323,7 +10414,7 @@
     <row r="16" spans="1:8" ht="12" customHeight="1">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
@@ -10335,7 +10426,7 @@
     <row r="17" spans="1:8" ht="12" customHeight="1">
       <c r="A17" s="1"/>
       <c r="B17" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>

</xml_diff>

<commit_message>
Versão do front-end 1.0.1
</commit_message>
<xml_diff>
--- a/01 - DB/Base_Pai_Troubleshooting_Alertas_Falhas_MVP.xlsx
+++ b/01 - DB/Base_Pai_Troubleshooting_Alertas_Falhas_MVP.xlsx
@@ -22,6 +22,7 @@
     <sheet name="Listas" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -2794,13 +2795,16 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2812,31 +2816,28 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3011,6 +3012,78 @@
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -3082,78 +3155,6 @@
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3168,51 +3169,51 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TabelaTroubleshooting" displayName="TabelaTroubleshooting" ref="A1:T194" headerRowDxfId="51" dataDxfId="50" totalsRowDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TabelaTroubleshooting" displayName="TabelaTroubleshooting" ref="A1:T194" headerRowDxfId="75" dataDxfId="74" totalsRowDxfId="73">
   <tableColumns count="20">
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Código" dataDxfId="48"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Tipo" dataDxfId="47"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Sistema" dataDxfId="46"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Subsistema" dataDxfId="45"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Severidade" dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Prioridade" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Status" dataDxfId="42"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Mensagem na IHM / Alerta" dataDxfId="41"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Descrição resumida" dataDxfId="40"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Causa" dataDxfId="39"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Efeito na máquina/operação" dataDxfId="38"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Solução" dataDxfId="37"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Validação após solução" dataDxfId="36"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Origem" dataDxfId="35"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Variável / Código relacionado" dataDxfId="34"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Ferramentas necessárias" dataDxfId="33"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Observações" dataDxfId="32"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Responsável" dataDxfId="31"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Data revisão" dataDxfId="30"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Versão" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Código" dataDxfId="72"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Tipo" dataDxfId="71"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Sistema" dataDxfId="70"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Subsistema" dataDxfId="69"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Severidade" dataDxfId="68"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Prioridade" dataDxfId="67"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Status" dataDxfId="66"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Mensagem na IHM / Alerta" dataDxfId="65"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Descrição resumida" dataDxfId="64"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Causa" dataDxfId="63"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Efeito na máquina/operação" dataDxfId="62"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Solução" dataDxfId="61"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Validação após solução" dataDxfId="60"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Origem" dataDxfId="59"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Variável / Código relacionado" dataDxfId="58"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Ferramentas necessárias" dataDxfId="57"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Observações" dataDxfId="56"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Responsável" dataDxfId="55"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Data revisão" dataDxfId="54"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Versão" dataDxfId="53"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{20343510-14AE-4192-A250-078DD82C5713}" name="TabelaDiagnosticoGuiado7" displayName="TabelaDiagnosticoGuiado7" ref="A1:O148" headerRowDxfId="75" dataDxfId="74" totalsRowDxfId="73">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{20343510-14AE-4192-A250-078DD82C5713}" name="TabelaDiagnosticoGuiado7" displayName="TabelaDiagnosticoGuiado7" ref="A1:O148" headerRowDxfId="52" dataDxfId="51" totalsRowDxfId="50">
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{63450B7D-49ED-41CF-B7D9-D287ED2CF298}" name="Código Item" dataDxfId="72"/>
-    <tableColumn id="4" xr3:uid="{46817399-D7BC-4925-942C-4CBCE861CEFB}" name="ID Passo" dataDxfId="71"/>
-    <tableColumn id="6" xr3:uid="{928114F4-FCAD-4C37-A4EF-819E9DF70EE8}" name="Nível" dataDxfId="70"/>
-    <tableColumn id="10" xr3:uid="{0D5C296C-DF81-40F3-8730-12258FC5A1C2}" name="Título do passo" dataDxfId="69"/>
-    <tableColumn id="13" xr3:uid="{C4B409B0-4E84-4D56-99DA-C47BE047C82F}" name="Condições" dataDxfId="68"/>
-    <tableColumn id="7" xr3:uid="{47B506C2-F1DC-4C47-B635-B1053D535C32}" name="Ação" dataDxfId="67"/>
-    <tableColumn id="8" xr3:uid="{9A1FD092-B7F8-4418-972E-572CF38F7734}" name="Especificação / Pergunta" dataDxfId="66"/>
-    <tableColumn id="12" xr3:uid="{79AF0F65-1615-411F-8D61-AF8DFB68EDBF}" name="Se SIM / OK" dataDxfId="65"/>
-    <tableColumn id="9" xr3:uid="{CE6BA67B-F888-46B1-8996-7107D16FBC60}" name="Se NÃO / NOK" dataDxfId="64"/>
-    <tableColumn id="2" xr3:uid="{22956E1A-E929-4E4C-96B4-A516DE98DA89}" name="Próximo passo SIM" dataDxfId="63" totalsRowDxfId="62"/>
-    <tableColumn id="3" xr3:uid="{D666DC4B-08B4-4658-ADE8-914DB4BD8A6F}" name="Próximo passo NÃO" dataDxfId="61" totalsRowDxfId="60"/>
-    <tableColumn id="5" xr3:uid="{6B4D0F42-A199-4F72-BCF8-87057820DA0B}" name="Reparo / Correção" dataDxfId="59" totalsRowDxfId="58"/>
-    <tableColumn id="11" xr3:uid="{B3E9C756-122E-4985-8678-E9E7E5C73523}" name="Ferramentas" dataDxfId="57" totalsRowDxfId="56"/>
-    <tableColumn id="14" xr3:uid="{98C258F9-4844-4EE4-A584-C7C40BA218E3}" name="Segurança" dataDxfId="55" totalsRowDxfId="54"/>
-    <tableColumn id="15" xr3:uid="{9450BD72-74B1-4478-982C-C7612EE8B7EC}" name="Observações" dataDxfId="53" totalsRowDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{63450B7D-49ED-41CF-B7D9-D287ED2CF298}" name="Código Item" dataDxfId="49"/>
+    <tableColumn id="4" xr3:uid="{46817399-D7BC-4925-942C-4CBCE861CEFB}" name="ID Passo" dataDxfId="48"/>
+    <tableColumn id="6" xr3:uid="{928114F4-FCAD-4C37-A4EF-819E9DF70EE8}" name="Nível" dataDxfId="47"/>
+    <tableColumn id="10" xr3:uid="{0D5C296C-DF81-40F3-8730-12258FC5A1C2}" name="Título do passo" dataDxfId="46"/>
+    <tableColumn id="13" xr3:uid="{C4B409B0-4E84-4D56-99DA-C47BE047C82F}" name="Condições" dataDxfId="45"/>
+    <tableColumn id="7" xr3:uid="{47B506C2-F1DC-4C47-B635-B1053D535C32}" name="Ação" dataDxfId="44"/>
+    <tableColumn id="8" xr3:uid="{9A1FD092-B7F8-4418-972E-572CF38F7734}" name="Especificação / Pergunta" dataDxfId="43"/>
+    <tableColumn id="12" xr3:uid="{79AF0F65-1615-411F-8D61-AF8DFB68EDBF}" name="Se SIM / OK" dataDxfId="42"/>
+    <tableColumn id="9" xr3:uid="{CE6BA67B-F888-46B1-8996-7107D16FBC60}" name="Se NÃO / NOK" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{22956E1A-E929-4E4C-96B4-A516DE98DA89}" name="Próximo passo SIM" dataDxfId="40" totalsRowDxfId="39"/>
+    <tableColumn id="3" xr3:uid="{D666DC4B-08B4-4658-ADE8-914DB4BD8A6F}" name="Próximo passo NÃO" dataDxfId="38" totalsRowDxfId="37"/>
+    <tableColumn id="5" xr3:uid="{6B4D0F42-A199-4F72-BCF8-87057820DA0B}" name="Reparo / Correção" dataDxfId="36" totalsRowDxfId="35"/>
+    <tableColumn id="11" xr3:uid="{B3E9C756-122E-4985-8678-E9E7E5C73523}" name="Ferramentas" dataDxfId="34" totalsRowDxfId="33"/>
+    <tableColumn id="14" xr3:uid="{98C258F9-4844-4EE4-A584-C7C40BA218E3}" name="Segurança" dataDxfId="32" totalsRowDxfId="31"/>
+    <tableColumn id="15" xr3:uid="{9450BD72-74B1-4478-982C-C7612EE8B7EC}" name="Observações" dataDxfId="30" totalsRowDxfId="29"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3434,31 +3435,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21.6" thickBot="1">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="19"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="28"/>
     </row>
     <row r="2" spans="1:8" ht="14.4" thickBot="1">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="23"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="29" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="24"/>
@@ -3470,40 +3471,40 @@
       <c r="H3" s="25"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="26" t="s">
+      <c r="A4" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="28"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="18"/>
     </row>
     <row r="5" spans="1:8" ht="14.4" thickBot="1">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="31"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" ht="14.4" thickBot="1">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="22"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="4" t="s">
@@ -3523,83 +3524,83 @@
       <c r="A8" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="28"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="18"/>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="27" t="s">
+      <c r="B9" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="27"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="28"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="18"/>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="27"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="28"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="18"/>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="28"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="18"/>
     </row>
     <row r="12" spans="1:8" ht="14.4" thickBot="1">
       <c r="A12" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="30" t="s">
+      <c r="B12" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="31"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="20"/>
     </row>
     <row r="13" spans="1:8" ht="14.4" thickBot="1">
-      <c r="A13" s="20" t="s">
+      <c r="A13" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="21"/>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
-      <c r="H13" s="22"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="23"/>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="4" t="s">
@@ -3619,85 +3620,85 @@
       <c r="A15" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="27" t="s">
+      <c r="B15" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="28"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="18"/>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="27" t="s">
+      <c r="B16" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="28"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="18"/>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="27"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="28"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="18"/>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="27" t="s">
+      <c r="B18" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="27"/>
-      <c r="D18" s="27"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="28"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="18"/>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="28"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="18"/>
     </row>
     <row r="20" spans="1:8" ht="14.4" thickBot="1">
       <c r="A20" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="30" t="s">
+      <c r="B20" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="31"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="20"/>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="3"/>
@@ -3721,26 +3722,26 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="B8:H8"/>
+    <mergeCell ref="B9:H9"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="B15:H15"/>
     <mergeCell ref="B16:H16"/>
     <mergeCell ref="B17:H17"/>
     <mergeCell ref="B18:H18"/>
     <mergeCell ref="B19:H19"/>
     <mergeCell ref="B20:H20"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B15:H15"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="B7:H7"/>
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="B9:H9"/>
-    <mergeCell ref="B10:H10"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A5:H5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8532,7 +8533,7 @@
     <col min="15" max="16384" width="47.5" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:15" ht="27.6">
       <c r="A1" s="3" t="s">
         <v>153</v>
       </c>
@@ -10130,7 +10131,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="35" spans="1:15" s="14" customFormat="1" ht="69">
+    <row r="35" spans="1:15" s="14" customFormat="1" ht="55.2">
       <c r="A35" s="3" t="s">
         <v>303</v>
       </c>
@@ -10459,7 +10460,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="42" spans="1:15" s="14" customFormat="1" ht="69">
+    <row r="42" spans="1:15" s="14" customFormat="1" ht="55.2">
       <c r="A42" s="3" t="s">
         <v>304</v>
       </c>
@@ -12010,7 +12011,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="75" spans="1:15" s="14" customFormat="1" ht="69">
+    <row r="75" spans="1:15" s="14" customFormat="1" ht="55.2">
       <c r="A75" s="14" t="s">
         <v>314</v>
       </c>

</xml_diff>